<commit_message>
Finalize DL comparison: MedViT1 small/base Final complete, final xlsx authoritative
</commit_message>
<xml_diff>
--- a/current_code_results/dl_supp/模型性能对比表_终版.xlsx
+++ b/current_code_results/dl_supp/模型性能对比表_终版.xlsx
@@ -1002,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1345,6 +1345,100 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>MedViT1-small</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Gray image 224^2</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>3 seeds</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0.759±0.017</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>0.693±0.097</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>0.680±0.089</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>0.640±0.052</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>0.795±0.072</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>0.635±0.274</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MedViT1-base</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Gray image 224^2</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>5 seeds</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.769±0.017</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0.486±0.222</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>0.857±0.089</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.654±0.042</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>0.810±0.021</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0.359±0.217</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1356,7 +1450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1477,88 +1571,88 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>MedViT1-small</t>
+          <t>ResNet50</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>BUSI</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.760 (仅s42)</t>
+          <t>0.923±0.010</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.760</t>
+          <t>0.925/0.934/0.910</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>⚠缺5 run</t>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>MedViT1-base</t>
+          <t>ConvNeXt-Tiny</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>internal</t>
+          <t>BUSI</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.942±0.012</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>0.924/0.951/0.949</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>未跑Final;best n5=0.773</t>
+          <t>✓</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ResNet50</t>
+          <t>MedViT1-small</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BUSI</t>
+          <t>internal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.923±0.010</t>
+          <t>0.759±0.017</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.925/0.934/0.910</t>
+          <t>0.760/0.737/0.780</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓ Final n3</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ConvNeXt-Tiny</t>
+          <t>MedViT1-small</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1568,17 +1662,71 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.942±0.012</t>
+          <t>0.898±0.019</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.924/0.951/0.949</t>
+          <t>0.872/0.918/0.903</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>✓</t>
+          <t>✓ Final n3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MedViT1-base</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>internal</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>0.769±0.017</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0.744/0.770/0.779/0.794/0.756</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>✓ Final n5</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>MedViT1-base</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>BUSI</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>0.941±0.008</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0.934/0.930/0.944/0.949/0.949</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>✓ Final n5</t>
         </is>
       </c>
     </row>

</xml_diff>